<commit_message>
Add Monthly Trend sheet with charts to BOM tracker
- 13 months (Jan-26 to Jan-27) with SUMPRODUCT formulas pulling from BOM Additions
- Columns: Month / # Additions / Total Value / Avg Value / Running Total
- Chart 1 (combo): qty bars (navy) + value line (amber) on dual axes
- Chart 2: cumulative value line (purple)
- All formulas update automatically as additions are entered
</commit_message>
<xml_diff>
--- a/BOM-Addition-Tracker.xlsx
+++ b/BOM-Addition-Tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet name="BOM Additions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Job Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Monthly Trend" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -149,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -273,6 +274,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -386,6 +402,365 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly BOM Additions — Qty &amp; Value</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Trend'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F3964"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1F3964"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Monthly Trend'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Trend'!$C$3:$C$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Trend'!D2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="25000">
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monthly Trend'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Trend'!$D$3:$D$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t># Additions</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Total Value (AUD)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumulative Value of BOM Additions (AUD)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Trend'!F2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="4B2D8B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="diamond"/>
+            <size val="5"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monthly Trend'!$A$3:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Trend'!$F$3:$F$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cumulative Value (AUD)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3340,4 +3715,431 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Monthly BOM Additions — Value &amp; Quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="22" t="inlineStr">
+        <is>
+          <t>Auto from BOM Additions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Month Start</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t># Additions</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Total Value (AUD)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Avg Value / Add.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Running Total AUD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="B3" s="44" t="n">
+        <v>46023</v>
+      </c>
+      <c r="C3" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B3))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B3))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D3" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B3))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B3))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E3" s="45">
+        <f>IF(C3=0,"",D3/C3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="45">
+        <f>D3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="n">
+        <v>46054</v>
+      </c>
+      <c r="C4" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B4))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B4))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D4" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B4))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B4))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E4" s="47">
+        <f>IF(C4=0,"",D4/C4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="47">
+        <f>F3+D4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C5" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B5))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B5))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D5" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B5))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B5))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E5" s="45">
+        <f>IF(C5=0,"",D5/C5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="45">
+        <f>F4+D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>46113</v>
+      </c>
+      <c r="C6" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B6))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B6))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D6" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B6))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B6))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E6" s="47">
+        <f>IF(C6=0,"",D6/C6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="47">
+        <f>F5+D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C7" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B7))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B7))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D7" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B7))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B7))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E7" s="45">
+        <f>IF(C7=0,"",D7/C7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="45">
+        <f>F6+D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>46174</v>
+      </c>
+      <c r="C8" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B8))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B8))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D8" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B8))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B8))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E8" s="47">
+        <f>IF(C8=0,"",D8/C8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="47">
+        <f>F7+D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C9" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B9))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B9))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D9" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B9))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B9))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E9" s="45">
+        <f>IF(C9=0,"",D9/C9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="45">
+        <f>F8+D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n">
+        <v>46235</v>
+      </c>
+      <c r="C10" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B10))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B10))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D10" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B10))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B10))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E10" s="47">
+        <f>IF(C10=0,"",D10/C10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="47">
+        <f>F9+D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="n">
+        <v>46266</v>
+      </c>
+      <c r="C11" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B11))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B11))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D11" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B11))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B11))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E11" s="45">
+        <f>IF(C11=0,"",D11/C11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="45">
+        <f>F10+D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C12" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B12))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B12))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B12))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B12))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E12" s="47">
+        <f>IF(C12=0,"",D12/C12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="47">
+        <f>F11+D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B13" s="44" t="n">
+        <v>46327</v>
+      </c>
+      <c r="C13" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B13))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B13))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D13" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B13))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B13))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E13" s="45">
+        <f>IF(C13=0,"",D13/C13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="45">
+        <f>F12+D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="n">
+        <v>46357</v>
+      </c>
+      <c r="C14" s="32">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B14))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B14))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D14" s="33">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B14))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B14))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E14" s="47">
+        <f>IF(C14=0,"",D14/C14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="47">
+        <f>F13+D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B15" s="44" t="n">
+        <v>46388</v>
+      </c>
+      <c r="C15" s="26">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B15))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B15))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
+        <v/>
+      </c>
+      <c r="D15" s="27">
+        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B15))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B15))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
+        <v/>
+      </c>
+      <c r="E15" s="45">
+        <f>IF(C15=0,"",D15/C15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="45">
+        <f>F14+D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>TOTALS</t>
+        </is>
+      </c>
+      <c r="C16" s="48">
+        <f>SUM(C3:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="39">
+        <f>SUM(D3:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="40" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="E1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Monthly Trend: Aug-26 to Jul-27, month labels on chart x-axis
- Changed period from Jan-26 to Aug-26 start (12 months: Aug-26 → Jul-27)
- Both charts now use month label column as x-axis categories
- Added axis number formats ($#,##0 on value axes, 0 on qty axis)
- Chart titles updated to reflect the date range
</commit_message>
<xml_diff>
--- a/BOM-Addition-Tracker.xlsx
+++ b/BOM-Addition-Tracker.xlsx
@@ -505,7 +505,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Monthly BOM Additions — Qty &amp; Value</a:t>
+              <a:t>Monthly BOM Additions — Quantity &amp; Value (Aug-26 to Jul-27)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -536,12 +536,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$15</f>
+              <f>'Monthly Trend'!$A$3:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$C$3:$C$15</f>
+              <f>'Monthly Trend'!$C$3:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -578,12 +578,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$15</f>
+              <f>'Monthly Trend'!$A$3:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$D$3:$D$15</f>
+              <f>'Monthly Trend'!$D$3:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -613,6 +613,7 @@
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -638,6 +639,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -664,6 +666,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -691,7 +694,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cumulative Value of BOM Additions (AUD)</a:t>
+              <a:t>Cumulative BOM Addition Cost (AUD) — Aug-26 to Jul-27</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -727,12 +730,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Monthly Trend'!$A$3:$A$15</f>
+              <f>'Monthly Trend'!$A$3:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly Trend'!$F$3:$F$15</f>
+              <f>'Monthly Trend'!$F$3:$F$14</f>
             </numRef>
           </val>
         </ser>
@@ -762,6 +765,7 @@
         </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -787,6 +791,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -807,10 +812,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="5040000"/>
+    <ext cx="8640000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -829,10 +834,10 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3600000"/>
+    <ext cx="8640000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -11305,7 +11310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11363,11 +11368,11 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>Jan-26</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="B3" s="61" t="n">
-        <v>46023</v>
+        <v>46235</v>
       </c>
       <c r="C3" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B3))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B3))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11389,11 +11394,11 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="32" t="inlineStr">
         <is>
-          <t>Feb-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="B4" s="62" t="n">
-        <v>46054</v>
+        <v>46266</v>
       </c>
       <c r="C4" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B4))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B4))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11415,11 +11420,11 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>Mar-26</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="B5" s="61" t="n">
-        <v>46082</v>
+        <v>46296</v>
       </c>
       <c r="C5" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B5))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B5))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11441,11 +11446,11 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="32" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="B6" s="62" t="n">
-        <v>46113</v>
+        <v>46327</v>
       </c>
       <c r="C6" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B6))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B6))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11467,11 +11472,11 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>May-26</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="B7" s="61" t="n">
-        <v>46143</v>
+        <v>46357</v>
       </c>
       <c r="C7" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B7))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B7))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11493,11 +11498,11 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="32" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="B8" s="62" t="n">
-        <v>46174</v>
+        <v>46388</v>
       </c>
       <c r="C8" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B8))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B8))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11519,11 +11524,11 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="B9" s="61" t="n">
-        <v>46204</v>
+        <v>46419</v>
       </c>
       <c r="C9" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B9))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B9))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11545,11 +11550,11 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="32" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="B10" s="62" t="n">
-        <v>46235</v>
+        <v>46447</v>
       </c>
       <c r="C10" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B10))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B10))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11571,11 +11576,11 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="B11" s="61" t="n">
-        <v>46266</v>
+        <v>46478</v>
       </c>
       <c r="C11" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B11))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B11))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11597,11 +11602,11 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="32" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="B12" s="62" t="n">
-        <v>46296</v>
+        <v>46508</v>
       </c>
       <c r="C12" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B12))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B12))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11623,11 +11628,11 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>Nov-26</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="B13" s="61" t="n">
-        <v>46327</v>
+        <v>46539</v>
       </c>
       <c r="C13" s="26">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B13))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B13))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11649,11 +11654,11 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="32" t="inlineStr">
         <is>
-          <t>Dec-26</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="B14" s="62" t="n">
-        <v>46357</v>
+        <v>46569</v>
       </c>
       <c r="C14" s="32">
         <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B14))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B14))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
@@ -11672,55 +11677,29 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>Jan-27</t>
-        </is>
-      </c>
-      <c r="B15" s="61" t="n">
-        <v>46388</v>
-      </c>
-      <c r="C15" s="26">
-        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B15))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B15))*ISNUMBER('BOM Additions'!$E$3:$E$53)*1)</f>
-        <v/>
-      </c>
-      <c r="D15" s="59">
-        <f>SUMPRODUCT((YEAR('BOM Additions'!$E$3:$E$53)=YEAR($B15))*(MONTH('BOM Additions'!$E$3:$E$53)=MONTH($B15))*ISNUMBER('BOM Additions'!$E$3:$E$53)*('BOM Additions'!$K$3:$K$53))</f>
-        <v/>
-      </c>
-      <c r="E15" s="52">
-        <f>IF(C15=0,"",D15/C15)</f>
-        <v/>
-      </c>
-      <c r="F15" s="52">
-        <f>F14+D15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="37" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B16" s="63" t="n"/>
-      <c r="C16" s="48">
-        <f>SUM(C3:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="64">
-        <f>SUM(D3:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="40" t="n"/>
-      <c r="F16" s="40" t="n"/>
+      <c r="B15" s="63" t="n"/>
+      <c r="C15" s="48">
+        <f>SUM(C3:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="64">
+        <f>SUM(D3:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="40" t="n"/>
+      <c r="F15" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A16:B16"/>
     <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix Days After Release formula — use INT() to prevent date formatting on date subtraction
</commit_message>
<xml_diff>
--- a/BOM-Addition-Tracker.xlsx
+++ b/BOM-Addition-Tracker.xlsx
@@ -1401,7 +1401,7 @@
       <c r="D4" s="51" t="n"/>
       <c r="E4" s="51" t="n"/>
       <c r="F4" s="13">
-        <f>IF(AND(D4&lt;&gt;"",E4&lt;&gt;""),E4-D4,"")</f>
+        <f>IF(AND(D4&lt;&gt;"",E4&lt;&gt;""),INT(E4)-INT(D4),"")</f>
         <v/>
       </c>
       <c r="G4" s="24" t="inlineStr">
@@ -1457,7 +1457,7 @@
       <c r="D5" s="53" t="n"/>
       <c r="E5" s="53" t="n"/>
       <c r="F5" s="18">
-        <f>IF(AND(D5&lt;&gt;"",E5&lt;&gt;""),E5-D5,"")</f>
+        <f>IF(AND(D5&lt;&gt;"",E5&lt;&gt;""),INT(E5)-INT(D5),"")</f>
         <v/>
       </c>
       <c r="G5" s="30" t="inlineStr">
@@ -1513,7 +1513,7 @@
       <c r="D6" s="51" t="n"/>
       <c r="E6" s="51" t="n"/>
       <c r="F6" s="13">
-        <f>IF(AND(D6&lt;&gt;"",E6&lt;&gt;""),E6-D6,"")</f>
+        <f>IF(AND(D6&lt;&gt;"",E6&lt;&gt;""),INT(E6)-INT(D6),"")</f>
         <v/>
       </c>
       <c r="G6" s="24" t="inlineStr">
@@ -1569,7 +1569,7 @@
       <c r="D7" s="53" t="n"/>
       <c r="E7" s="53" t="n"/>
       <c r="F7" s="18">
-        <f>IF(AND(D7&lt;&gt;"",E7&lt;&gt;""),E7-D7,"")</f>
+        <f>IF(AND(D7&lt;&gt;"",E7&lt;&gt;""),INT(E7)-INT(D7),"")</f>
         <v/>
       </c>
       <c r="G7" s="30" t="inlineStr">
@@ -1625,7 +1625,7 @@
       <c r="D8" s="51" t="n"/>
       <c r="E8" s="51" t="n"/>
       <c r="F8" s="13">
-        <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),E8-D8,"")</f>
+        <f>IF(AND(D8&lt;&gt;"",E8&lt;&gt;""),INT(E8)-INT(D8),"")</f>
         <v/>
       </c>
       <c r="G8" s="24" t="inlineStr">
@@ -1681,7 +1681,7 @@
       <c r="D9" s="53" t="n"/>
       <c r="E9" s="53" t="n"/>
       <c r="F9" s="18">
-        <f>IF(AND(D9&lt;&gt;"",E9&lt;&gt;""),E9-D9,"")</f>
+        <f>IF(AND(D9&lt;&gt;"",E9&lt;&gt;""),INT(E9)-INT(D9),"")</f>
         <v/>
       </c>
       <c r="G9" s="30" t="inlineStr">
@@ -1737,7 +1737,7 @@
       <c r="D10" s="51" t="n"/>
       <c r="E10" s="51" t="n"/>
       <c r="F10" s="13">
-        <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),E10-D10,"")</f>
+        <f>IF(AND(D10&lt;&gt;"",E10&lt;&gt;""),INT(E10)-INT(D10),"")</f>
         <v/>
       </c>
       <c r="G10" s="24" t="inlineStr">
@@ -1793,7 +1793,7 @@
       <c r="D11" s="53" t="n"/>
       <c r="E11" s="53" t="n"/>
       <c r="F11" s="18">
-        <f>IF(AND(D11&lt;&gt;"",E11&lt;&gt;""),E11-D11,"")</f>
+        <f>IF(AND(D11&lt;&gt;"",E11&lt;&gt;""),INT(E11)-INT(D11),"")</f>
         <v/>
       </c>
       <c r="G11" s="30" t="inlineStr">
@@ -1849,7 +1849,7 @@
       <c r="D12" s="51" t="n"/>
       <c r="E12" s="51" t="n"/>
       <c r="F12" s="13">
-        <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),E12-D12,"")</f>
+        <f>IF(AND(D12&lt;&gt;"",E12&lt;&gt;""),INT(E12)-INT(D12),"")</f>
         <v/>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -1917,7 +1917,7 @@
       <c r="D13" s="53" t="n"/>
       <c r="E13" s="53" t="n"/>
       <c r="F13" s="18">
-        <f>IF(AND(D13&lt;&gt;"",E13&lt;&gt;""),E13-D13,"")</f>
+        <f>IF(AND(D13&lt;&gt;"",E13&lt;&gt;""),INT(E13)-INT(D13),"")</f>
         <v/>
       </c>
       <c r="G13" s="30" t="inlineStr">
@@ -1985,7 +1985,7 @@
       <c r="D14" s="51" t="n"/>
       <c r="E14" s="51" t="n"/>
       <c r="F14" s="13">
-        <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),E14-D14,"")</f>
+        <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),INT(E14)-INT(D14),"")</f>
         <v/>
       </c>
       <c r="G14" s="24" t="inlineStr">
@@ -2053,7 +2053,7 @@
       <c r="D15" s="53" t="n"/>
       <c r="E15" s="53" t="n"/>
       <c r="F15" s="18">
-        <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),E15-D15,"")</f>
+        <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),INT(E15)-INT(D15),"")</f>
         <v/>
       </c>
       <c r="G15" s="30" t="inlineStr">
@@ -2121,7 +2121,7 @@
       <c r="D16" s="51" t="n"/>
       <c r="E16" s="51" t="n"/>
       <c r="F16" s="13">
-        <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),E16-D16,"")</f>
+        <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),INT(E16)-INT(D16),"")</f>
         <v/>
       </c>
       <c r="G16" s="24" t="inlineStr">
@@ -2189,7 +2189,7 @@
       <c r="D17" s="53" t="n"/>
       <c r="E17" s="53" t="n"/>
       <c r="F17" s="18">
-        <f>IF(AND(D17&lt;&gt;"",E17&lt;&gt;""),E17-D17,"")</f>
+        <f>IF(AND(D17&lt;&gt;"",E17&lt;&gt;""),INT(E17)-INT(D17),"")</f>
         <v/>
       </c>
       <c r="G17" s="30" t="inlineStr">
@@ -2257,7 +2257,7 @@
       <c r="D18" s="51" t="n"/>
       <c r="E18" s="51" t="n"/>
       <c r="F18" s="13">
-        <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),E18-D18,"")</f>
+        <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),INT(E18)-INT(D18),"")</f>
         <v/>
       </c>
       <c r="G18" s="24" t="inlineStr">
@@ -2325,7 +2325,7 @@
       <c r="D19" s="53" t="n"/>
       <c r="E19" s="53" t="n"/>
       <c r="F19" s="18">
-        <f>IF(AND(D19&lt;&gt;"",E19&lt;&gt;""),E19-D19,"")</f>
+        <f>IF(AND(D19&lt;&gt;"",E19&lt;&gt;""),INT(E19)-INT(D19),"")</f>
         <v/>
       </c>
       <c r="G19" s="30" t="inlineStr">
@@ -2393,7 +2393,7 @@
       <c r="D20" s="51" t="n"/>
       <c r="E20" s="51" t="n"/>
       <c r="F20" s="13">
-        <f>IF(AND(D20&lt;&gt;"",E20&lt;&gt;""),E20-D20,"")</f>
+        <f>IF(AND(D20&lt;&gt;"",E20&lt;&gt;""),INT(E20)-INT(D20),"")</f>
         <v/>
       </c>
       <c r="G20" s="24" t="inlineStr">
@@ -2461,7 +2461,7 @@
       <c r="D21" s="53" t="n"/>
       <c r="E21" s="53" t="n"/>
       <c r="F21" s="18">
-        <f>IF(AND(D21&lt;&gt;"",E21&lt;&gt;""),E21-D21,"")</f>
+        <f>IF(AND(D21&lt;&gt;"",E21&lt;&gt;""),INT(E21)-INT(D21),"")</f>
         <v/>
       </c>
       <c r="G21" s="30" t="inlineStr">
@@ -2525,7 +2525,7 @@
       <c r="D22" s="51" t="n"/>
       <c r="E22" s="51" t="n"/>
       <c r="F22" s="13">
-        <f>IF(AND(D22&lt;&gt;"",E22&lt;&gt;""),E22-D22,"")</f>
+        <f>IF(AND(D22&lt;&gt;"",E22&lt;&gt;""),INT(E22)-INT(D22),"")</f>
         <v/>
       </c>
       <c r="G22" s="24" t="inlineStr">
@@ -2589,7 +2589,7 @@
       <c r="D23" s="53" t="n"/>
       <c r="E23" s="53" t="n"/>
       <c r="F23" s="18">
-        <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),E23-D23,"")</f>
+        <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),INT(E23)-INT(D23),"")</f>
         <v/>
       </c>
       <c r="G23" s="30" t="inlineStr">
@@ -2653,7 +2653,7 @@
       <c r="D24" s="51" t="n"/>
       <c r="E24" s="51" t="n"/>
       <c r="F24" s="13">
-        <f>IF(AND(D24&lt;&gt;"",E24&lt;&gt;""),E24-D24,"")</f>
+        <f>IF(AND(D24&lt;&gt;"",E24&lt;&gt;""),INT(E24)-INT(D24),"")</f>
         <v/>
       </c>
       <c r="G24" s="24" t="inlineStr">
@@ -2717,7 +2717,7 @@
       <c r="D25" s="53" t="n"/>
       <c r="E25" s="53" t="n"/>
       <c r="F25" s="18">
-        <f>IF(AND(D25&lt;&gt;"",E25&lt;&gt;""),E25-D25,"")</f>
+        <f>IF(AND(D25&lt;&gt;"",E25&lt;&gt;""),INT(E25)-INT(D25),"")</f>
         <v/>
       </c>
       <c r="G25" s="30" t="inlineStr">
@@ -2781,7 +2781,7 @@
       <c r="D26" s="51" t="n"/>
       <c r="E26" s="51" t="n"/>
       <c r="F26" s="13">
-        <f>IF(AND(D26&lt;&gt;"",E26&lt;&gt;""),E26-D26,"")</f>
+        <f>IF(AND(D26&lt;&gt;"",E26&lt;&gt;""),INT(E26)-INT(D26),"")</f>
         <v/>
       </c>
       <c r="G26" s="24" t="inlineStr">
@@ -2845,7 +2845,7 @@
       <c r="D27" s="53" t="n"/>
       <c r="E27" s="53" t="n"/>
       <c r="F27" s="18">
-        <f>IF(AND(D27&lt;&gt;"",E27&lt;&gt;""),E27-D27,"")</f>
+        <f>IF(AND(D27&lt;&gt;"",E27&lt;&gt;""),INT(E27)-INT(D27),"")</f>
         <v/>
       </c>
       <c r="G27" s="30" t="inlineStr">
@@ -2909,7 +2909,7 @@
       <c r="D28" s="51" t="n"/>
       <c r="E28" s="51" t="n"/>
       <c r="F28" s="13">
-        <f>IF(AND(D28&lt;&gt;"",E28&lt;&gt;""),E28-D28,"")</f>
+        <f>IF(AND(D28&lt;&gt;"",E28&lt;&gt;""),INT(E28)-INT(D28),"")</f>
         <v/>
       </c>
       <c r="G28" s="24" t="inlineStr">
@@ -2973,7 +2973,7 @@
       <c r="D29" s="53" t="n"/>
       <c r="E29" s="53" t="n"/>
       <c r="F29" s="18">
-        <f>IF(AND(D29&lt;&gt;"",E29&lt;&gt;""),E29-D29,"")</f>
+        <f>IF(AND(D29&lt;&gt;"",E29&lt;&gt;""),INT(E29)-INT(D29),"")</f>
         <v/>
       </c>
       <c r="G29" s="30" t="inlineStr">
@@ -3037,7 +3037,7 @@
       <c r="D30" s="51" t="n"/>
       <c r="E30" s="51" t="n"/>
       <c r="F30" s="13">
-        <f>IF(AND(D30&lt;&gt;"",E30&lt;&gt;""),E30-D30,"")</f>
+        <f>IF(AND(D30&lt;&gt;"",E30&lt;&gt;""),INT(E30)-INT(D30),"")</f>
         <v/>
       </c>
       <c r="G30" s="24" t="inlineStr">
@@ -3101,7 +3101,7 @@
       <c r="D31" s="53" t="n"/>
       <c r="E31" s="53" t="n"/>
       <c r="F31" s="18">
-        <f>IF(AND(D31&lt;&gt;"",E31&lt;&gt;""),E31-D31,"")</f>
+        <f>IF(AND(D31&lt;&gt;"",E31&lt;&gt;""),INT(E31)-INT(D31),"")</f>
         <v/>
       </c>
       <c r="G31" s="30" t="inlineStr">
@@ -3165,7 +3165,7 @@
       <c r="D32" s="51" t="n"/>
       <c r="E32" s="51" t="n"/>
       <c r="F32" s="13">
-        <f>IF(AND(D32&lt;&gt;"",E32&lt;&gt;""),E32-D32,"")</f>
+        <f>IF(AND(D32&lt;&gt;"",E32&lt;&gt;""),INT(E32)-INT(D32),"")</f>
         <v/>
       </c>
       <c r="G32" s="24" t="inlineStr">
@@ -3229,7 +3229,7 @@
       <c r="D33" s="53" t="n"/>
       <c r="E33" s="53" t="n"/>
       <c r="F33" s="18">
-        <f>IF(AND(D33&lt;&gt;"",E33&lt;&gt;""),E33-D33,"")</f>
+        <f>IF(AND(D33&lt;&gt;"",E33&lt;&gt;""),INT(E33)-INT(D33),"")</f>
         <v/>
       </c>
       <c r="G33" s="30" t="inlineStr">
@@ -3293,7 +3293,7 @@
       <c r="D34" s="51" t="n"/>
       <c r="E34" s="51" t="n"/>
       <c r="F34" s="13">
-        <f>IF(AND(D34&lt;&gt;"",E34&lt;&gt;""),E34-D34,"")</f>
+        <f>IF(AND(D34&lt;&gt;"",E34&lt;&gt;""),INT(E34)-INT(D34),"")</f>
         <v/>
       </c>
       <c r="G34" s="24" t="inlineStr">
@@ -3357,7 +3357,7 @@
       <c r="D35" s="53" t="n"/>
       <c r="E35" s="53" t="n"/>
       <c r="F35" s="18">
-        <f>IF(AND(D35&lt;&gt;"",E35&lt;&gt;""),E35-D35,"")</f>
+        <f>IF(AND(D35&lt;&gt;"",E35&lt;&gt;""),INT(E35)-INT(D35),"")</f>
         <v/>
       </c>
       <c r="G35" s="30" t="inlineStr">
@@ -3425,7 +3425,7 @@
       <c r="D36" s="51" t="n"/>
       <c r="E36" s="51" t="n"/>
       <c r="F36" s="13">
-        <f>IF(AND(D36&lt;&gt;"",E36&lt;&gt;""),E36-D36,"")</f>
+        <f>IF(AND(D36&lt;&gt;"",E36&lt;&gt;""),INT(E36)-INT(D36),"")</f>
         <v/>
       </c>
       <c r="G36" s="24" t="inlineStr">
@@ -3489,7 +3489,7 @@
       <c r="D37" s="53" t="n"/>
       <c r="E37" s="53" t="n"/>
       <c r="F37" s="18">
-        <f>IF(AND(D37&lt;&gt;"",E37&lt;&gt;""),E37-D37,"")</f>
+        <f>IF(AND(D37&lt;&gt;"",E37&lt;&gt;""),INT(E37)-INT(D37),"")</f>
         <v/>
       </c>
       <c r="G37" s="30" t="inlineStr">
@@ -3553,7 +3553,7 @@
       <c r="D38" s="51" t="n"/>
       <c r="E38" s="51" t="n"/>
       <c r="F38" s="13">
-        <f>IF(AND(D38&lt;&gt;"",E38&lt;&gt;""),E38-D38,"")</f>
+        <f>IF(AND(D38&lt;&gt;"",E38&lt;&gt;""),INT(E38)-INT(D38),"")</f>
         <v/>
       </c>
       <c r="G38" s="24" t="inlineStr">
@@ -3617,7 +3617,7 @@
       <c r="D39" s="53" t="n"/>
       <c r="E39" s="53" t="n"/>
       <c r="F39" s="18">
-        <f>IF(AND(D39&lt;&gt;"",E39&lt;&gt;""),E39-D39,"")</f>
+        <f>IF(AND(D39&lt;&gt;"",E39&lt;&gt;""),INT(E39)-INT(D39),"")</f>
         <v/>
       </c>
       <c r="G39" s="30" t="inlineStr">
@@ -3683,7 +3683,7 @@
       <c r="D40" s="51" t="n"/>
       <c r="E40" s="51" t="n"/>
       <c r="F40" s="13">
-        <f>IF(AND(D40&lt;&gt;"",E40&lt;&gt;""),E40-D40,"")</f>
+        <f>IF(AND(D40&lt;&gt;"",E40&lt;&gt;""),INT(E40)-INT(D40),"")</f>
         <v/>
       </c>
       <c r="G40" s="24" t="inlineStr">
@@ -3749,7 +3749,7 @@
       <c r="D41" s="53" t="n"/>
       <c r="E41" s="53" t="n"/>
       <c r="F41" s="18">
-        <f>IF(AND(D41&lt;&gt;"",E41&lt;&gt;""),E41-D41,"")</f>
+        <f>IF(AND(D41&lt;&gt;"",E41&lt;&gt;""),INT(E41)-INT(D41),"")</f>
         <v/>
       </c>
       <c r="G41" s="30" t="inlineStr">
@@ -3815,7 +3815,7 @@
       <c r="D42" s="51" t="n"/>
       <c r="E42" s="51" t="n"/>
       <c r="F42" s="13">
-        <f>IF(AND(D42&lt;&gt;"",E42&lt;&gt;""),E42-D42,"")</f>
+        <f>IF(AND(D42&lt;&gt;"",E42&lt;&gt;""),INT(E42)-INT(D42),"")</f>
         <v/>
       </c>
       <c r="G42" s="24" t="inlineStr">
@@ -3879,7 +3879,7 @@
       <c r="D43" s="53" t="n"/>
       <c r="E43" s="53" t="n"/>
       <c r="F43" s="18">
-        <f>IF(AND(D43&lt;&gt;"",E43&lt;&gt;""),E43-D43,"")</f>
+        <f>IF(AND(D43&lt;&gt;"",E43&lt;&gt;""),INT(E43)-INT(D43),"")</f>
         <v/>
       </c>
       <c r="G43" s="30" t="inlineStr">
@@ -3943,7 +3943,7 @@
       <c r="D44" s="51" t="n"/>
       <c r="E44" s="51" t="n"/>
       <c r="F44" s="13">
-        <f>IF(AND(D44&lt;&gt;"",E44&lt;&gt;""),E44-D44,"")</f>
+        <f>IF(AND(D44&lt;&gt;"",E44&lt;&gt;""),INT(E44)-INT(D44),"")</f>
         <v/>
       </c>
       <c r="G44" s="24" t="inlineStr">
@@ -4007,7 +4007,7 @@
       <c r="D45" s="53" t="n"/>
       <c r="E45" s="53" t="n"/>
       <c r="F45" s="18">
-        <f>IF(AND(D45&lt;&gt;"",E45&lt;&gt;""),E45-D45,"")</f>
+        <f>IF(AND(D45&lt;&gt;"",E45&lt;&gt;""),INT(E45)-INT(D45),"")</f>
         <v/>
       </c>
       <c r="G45" s="30" t="inlineStr">
@@ -4071,7 +4071,7 @@
       <c r="D46" s="51" t="n"/>
       <c r="E46" s="51" t="n"/>
       <c r="F46" s="13">
-        <f>IF(AND(D46&lt;&gt;"",E46&lt;&gt;""),E46-D46,"")</f>
+        <f>IF(AND(D46&lt;&gt;"",E46&lt;&gt;""),INT(E46)-INT(D46),"")</f>
         <v/>
       </c>
       <c r="G46" s="24" t="inlineStr">
@@ -4135,7 +4135,7 @@
       <c r="D47" s="53" t="n"/>
       <c r="E47" s="53" t="n"/>
       <c r="F47" s="18">
-        <f>IF(AND(D47&lt;&gt;"",E47&lt;&gt;""),E47-D47,"")</f>
+        <f>IF(AND(D47&lt;&gt;"",E47&lt;&gt;""),INT(E47)-INT(D47),"")</f>
         <v/>
       </c>
       <c r="G47" s="30" t="inlineStr">
@@ -4199,7 +4199,7 @@
       <c r="D48" s="51" t="n"/>
       <c r="E48" s="51" t="n"/>
       <c r="F48" s="13">
-        <f>IF(AND(D48&lt;&gt;"",E48&lt;&gt;""),E48-D48,"")</f>
+        <f>IF(AND(D48&lt;&gt;"",E48&lt;&gt;""),INT(E48)-INT(D48),"")</f>
         <v/>
       </c>
       <c r="G48" s="24" t="inlineStr">
@@ -4263,7 +4263,7 @@
       <c r="D49" s="53" t="n"/>
       <c r="E49" s="53" t="n"/>
       <c r="F49" s="18">
-        <f>IF(AND(D49&lt;&gt;"",E49&lt;&gt;""),E49-D49,"")</f>
+        <f>IF(AND(D49&lt;&gt;"",E49&lt;&gt;""),INT(E49)-INT(D49),"")</f>
         <v/>
       </c>
       <c r="G49" s="30" t="inlineStr">
@@ -4327,7 +4327,7 @@
       <c r="D50" s="51" t="n"/>
       <c r="E50" s="51" t="n"/>
       <c r="F50" s="13">
-        <f>IF(AND(D50&lt;&gt;"",E50&lt;&gt;""),E50-D50,"")</f>
+        <f>IF(AND(D50&lt;&gt;"",E50&lt;&gt;""),INT(E50)-INT(D50),"")</f>
         <v/>
       </c>
       <c r="G50" s="24" t="inlineStr">
@@ -4391,7 +4391,7 @@
       <c r="D51" s="53" t="n"/>
       <c r="E51" s="53" t="n"/>
       <c r="F51" s="18">
-        <f>IF(AND(D51&lt;&gt;"",E51&lt;&gt;""),E51-D51,"")</f>
+        <f>IF(AND(D51&lt;&gt;"",E51&lt;&gt;""),INT(E51)-INT(D51),"")</f>
         <v/>
       </c>
       <c r="G51" s="30" t="inlineStr">
@@ -4457,7 +4457,7 @@
       <c r="D52" s="51" t="n"/>
       <c r="E52" s="51" t="n"/>
       <c r="F52" s="13">
-        <f>IF(AND(D52&lt;&gt;"",E52&lt;&gt;""),E52-D52,"")</f>
+        <f>IF(AND(D52&lt;&gt;"",E52&lt;&gt;""),INT(E52)-INT(D52),"")</f>
         <v/>
       </c>
       <c r="G52" s="24" t="inlineStr">
@@ -4523,7 +4523,7 @@
       <c r="D53" s="53" t="n"/>
       <c r="E53" s="53" t="n"/>
       <c r="F53" s="18">
-        <f>IF(AND(D53&lt;&gt;"",E53&lt;&gt;""),E53-D53,"")</f>
+        <f>IF(AND(D53&lt;&gt;"",E53&lt;&gt;""),INT(E53)-INT(D53),"")</f>
         <v/>
       </c>
       <c r="G53" s="30" t="inlineStr">
@@ -4589,7 +4589,7 @@
       <c r="D54" s="51" t="n"/>
       <c r="E54" s="51" t="n"/>
       <c r="F54" s="13">
-        <f>IF(AND(D54&lt;&gt;"",E54&lt;&gt;""),E54-D54,"")</f>
+        <f>IF(AND(D54&lt;&gt;"",E54&lt;&gt;""),INT(E54)-INT(D54),"")</f>
         <v/>
       </c>
       <c r="G54" s="24" t="inlineStr">
@@ -4655,7 +4655,7 @@
       <c r="D55" s="53" t="n"/>
       <c r="E55" s="53" t="n"/>
       <c r="F55" s="18">
-        <f>IF(AND(D55&lt;&gt;"",E55&lt;&gt;""),E55-D55,"")</f>
+        <f>IF(AND(D55&lt;&gt;"",E55&lt;&gt;""),INT(E55)-INT(D55),"")</f>
         <v/>
       </c>
       <c r="G55" s="30" t="inlineStr">
@@ -4721,7 +4721,7 @@
       <c r="D56" s="51" t="n"/>
       <c r="E56" s="51" t="n"/>
       <c r="F56" s="13">
-        <f>IF(AND(D56&lt;&gt;"",E56&lt;&gt;""),E56-D56,"")</f>
+        <f>IF(AND(D56&lt;&gt;"",E56&lt;&gt;""),INT(E56)-INT(D56),"")</f>
         <v/>
       </c>
       <c r="G56" s="24" t="inlineStr">
@@ -4787,7 +4787,7 @@
       <c r="D57" s="53" t="n"/>
       <c r="E57" s="53" t="n"/>
       <c r="F57" s="18">
-        <f>IF(AND(D57&lt;&gt;"",E57&lt;&gt;""),E57-D57,"")</f>
+        <f>IF(AND(D57&lt;&gt;"",E57&lt;&gt;""),INT(E57)-INT(D57),"")</f>
         <v/>
       </c>
       <c r="G57" s="30" t="inlineStr">
@@ -4853,7 +4853,7 @@
       <c r="D58" s="51" t="n"/>
       <c r="E58" s="51" t="n"/>
       <c r="F58" s="13">
-        <f>IF(AND(D58&lt;&gt;"",E58&lt;&gt;""),E58-D58,"")</f>
+        <f>IF(AND(D58&lt;&gt;"",E58&lt;&gt;""),INT(E58)-INT(D58),"")</f>
         <v/>
       </c>
       <c r="G58" s="24" t="inlineStr">
@@ -4921,7 +4921,7 @@
       <c r="D59" s="53" t="n"/>
       <c r="E59" s="53" t="n"/>
       <c r="F59" s="18">
-        <f>IF(AND(D59&lt;&gt;"",E59&lt;&gt;""),E59-D59,"")</f>
+        <f>IF(AND(D59&lt;&gt;"",E59&lt;&gt;""),INT(E59)-INT(D59),"")</f>
         <v/>
       </c>
       <c r="G59" s="30" t="inlineStr">
@@ -4989,7 +4989,7 @@
       <c r="D60" s="51" t="n"/>
       <c r="E60" s="51" t="n"/>
       <c r="F60" s="13">
-        <f>IF(AND(D60&lt;&gt;"",E60&lt;&gt;""),E60-D60,"")</f>
+        <f>IF(AND(D60&lt;&gt;"",E60&lt;&gt;""),INT(E60)-INT(D60),"")</f>
         <v/>
       </c>
       <c r="G60" s="24" t="inlineStr">
@@ -5057,7 +5057,7 @@
       <c r="D61" s="53" t="n"/>
       <c r="E61" s="53" t="n"/>
       <c r="F61" s="18">
-        <f>IF(AND(D61&lt;&gt;"",E61&lt;&gt;""),E61-D61,"")</f>
+        <f>IF(AND(D61&lt;&gt;"",E61&lt;&gt;""),INT(E61)-INT(D61),"")</f>
         <v/>
       </c>
       <c r="G61" s="30" t="inlineStr">
@@ -5125,7 +5125,7 @@
       <c r="D62" s="51" t="n"/>
       <c r="E62" s="51" t="n"/>
       <c r="F62" s="13">
-        <f>IF(AND(D62&lt;&gt;"",E62&lt;&gt;""),E62-D62,"")</f>
+        <f>IF(AND(D62&lt;&gt;"",E62&lt;&gt;""),INT(E62)-INT(D62),"")</f>
         <v/>
       </c>
       <c r="G62" s="24" t="inlineStr">
@@ -5193,7 +5193,7 @@
       <c r="D63" s="53" t="n"/>
       <c r="E63" s="53" t="n"/>
       <c r="F63" s="18">
-        <f>IF(AND(D63&lt;&gt;"",E63&lt;&gt;""),E63-D63,"")</f>
+        <f>IF(AND(D63&lt;&gt;"",E63&lt;&gt;""),INT(E63)-INT(D63),"")</f>
         <v/>
       </c>
       <c r="G63" s="30" t="inlineStr">
@@ -5261,7 +5261,7 @@
       <c r="D64" s="51" t="n"/>
       <c r="E64" s="51" t="n"/>
       <c r="F64" s="13">
-        <f>IF(AND(D64&lt;&gt;"",E64&lt;&gt;""),E64-D64,"")</f>
+        <f>IF(AND(D64&lt;&gt;"",E64&lt;&gt;""),INT(E64)-INT(D64),"")</f>
         <v/>
       </c>
       <c r="G64" s="24" t="inlineStr">
@@ -5329,7 +5329,7 @@
       <c r="D65" s="53" t="n"/>
       <c r="E65" s="53" t="n"/>
       <c r="F65" s="18">
-        <f>IF(AND(D65&lt;&gt;"",E65&lt;&gt;""),E65-D65,"")</f>
+        <f>IF(AND(D65&lt;&gt;"",E65&lt;&gt;""),INT(E65)-INT(D65),"")</f>
         <v/>
       </c>
       <c r="G65" s="30" t="inlineStr">
@@ -5397,7 +5397,7 @@
       <c r="D66" s="51" t="n"/>
       <c r="E66" s="51" t="n"/>
       <c r="F66" s="13">
-        <f>IF(AND(D66&lt;&gt;"",E66&lt;&gt;""),E66-D66,"")</f>
+        <f>IF(AND(D66&lt;&gt;"",E66&lt;&gt;""),INT(E66)-INT(D66),"")</f>
         <v/>
       </c>
       <c r="G66" s="24" t="inlineStr">
@@ -5465,7 +5465,7 @@
       <c r="D67" s="53" t="n"/>
       <c r="E67" s="53" t="n"/>
       <c r="F67" s="18">
-        <f>IF(AND(D67&lt;&gt;"",E67&lt;&gt;""),E67-D67,"")</f>
+        <f>IF(AND(D67&lt;&gt;"",E67&lt;&gt;""),INT(E67)-INT(D67),"")</f>
         <v/>
       </c>
       <c r="G67" s="30" t="inlineStr">
@@ -5533,7 +5533,7 @@
       <c r="D68" s="51" t="n"/>
       <c r="E68" s="51" t="n"/>
       <c r="F68" s="13">
-        <f>IF(AND(D68&lt;&gt;"",E68&lt;&gt;""),E68-D68,"")</f>
+        <f>IF(AND(D68&lt;&gt;"",E68&lt;&gt;""),INT(E68)-INT(D68),"")</f>
         <v/>
       </c>
       <c r="G68" s="24" t="inlineStr">
@@ -5601,7 +5601,7 @@
       <c r="D69" s="53" t="n"/>
       <c r="E69" s="53" t="n"/>
       <c r="F69" s="18">
-        <f>IF(AND(D69&lt;&gt;"",E69&lt;&gt;""),E69-D69,"")</f>
+        <f>IF(AND(D69&lt;&gt;"",E69&lt;&gt;""),INT(E69)-INT(D69),"")</f>
         <v/>
       </c>
       <c r="G69" s="30" t="inlineStr">
@@ -5669,7 +5669,7 @@
       <c r="D70" s="51" t="n"/>
       <c r="E70" s="51" t="n"/>
       <c r="F70" s="13">
-        <f>IF(AND(D70&lt;&gt;"",E70&lt;&gt;""),E70-D70,"")</f>
+        <f>IF(AND(D70&lt;&gt;"",E70&lt;&gt;""),INT(E70)-INT(D70),"")</f>
         <v/>
       </c>
       <c r="G70" s="24" t="inlineStr">
@@ -5737,7 +5737,7 @@
       <c r="D71" s="53" t="n"/>
       <c r="E71" s="53" t="n"/>
       <c r="F71" s="18">
-        <f>IF(AND(D71&lt;&gt;"",E71&lt;&gt;""),E71-D71,"")</f>
+        <f>IF(AND(D71&lt;&gt;"",E71&lt;&gt;""),INT(E71)-INT(D71),"")</f>
         <v/>
       </c>
       <c r="G71" s="30" t="inlineStr">
@@ -5805,7 +5805,7 @@
       <c r="D72" s="51" t="n"/>
       <c r="E72" s="51" t="n"/>
       <c r="F72" s="13">
-        <f>IF(AND(D72&lt;&gt;"",E72&lt;&gt;""),E72-D72,"")</f>
+        <f>IF(AND(D72&lt;&gt;"",E72&lt;&gt;""),INT(E72)-INT(D72),"")</f>
         <v/>
       </c>
       <c r="G72" s="24" t="inlineStr">
@@ -5873,7 +5873,7 @@
       <c r="D73" s="53" t="n"/>
       <c r="E73" s="53" t="n"/>
       <c r="F73" s="18">
-        <f>IF(AND(D73&lt;&gt;"",E73&lt;&gt;""),E73-D73,"")</f>
+        <f>IF(AND(D73&lt;&gt;"",E73&lt;&gt;""),INT(E73)-INT(D73),"")</f>
         <v/>
       </c>
       <c r="G73" s="30" t="inlineStr">
@@ -5941,7 +5941,7 @@
       <c r="D74" s="51" t="n"/>
       <c r="E74" s="51" t="n"/>
       <c r="F74" s="13">
-        <f>IF(AND(D74&lt;&gt;"",E74&lt;&gt;""),E74-D74,"")</f>
+        <f>IF(AND(D74&lt;&gt;"",E74&lt;&gt;""),INT(E74)-INT(D74),"")</f>
         <v/>
       </c>
       <c r="G74" s="24" t="inlineStr">
@@ -6009,7 +6009,7 @@
       <c r="D75" s="53" t="n"/>
       <c r="E75" s="53" t="n"/>
       <c r="F75" s="18">
-        <f>IF(AND(D75&lt;&gt;"",E75&lt;&gt;""),E75-D75,"")</f>
+        <f>IF(AND(D75&lt;&gt;"",E75&lt;&gt;""),INT(E75)-INT(D75),"")</f>
         <v/>
       </c>
       <c r="G75" s="30" t="inlineStr">
@@ -6077,7 +6077,7 @@
       <c r="D76" s="51" t="n"/>
       <c r="E76" s="51" t="n"/>
       <c r="F76" s="13">
-        <f>IF(AND(D76&lt;&gt;"",E76&lt;&gt;""),E76-D76,"")</f>
+        <f>IF(AND(D76&lt;&gt;"",E76&lt;&gt;""),INT(E76)-INT(D76),"")</f>
         <v/>
       </c>
       <c r="G76" s="24" t="inlineStr">
@@ -6141,7 +6141,7 @@
       <c r="D77" s="53" t="n"/>
       <c r="E77" s="53" t="n"/>
       <c r="F77" s="18">
-        <f>IF(AND(D77&lt;&gt;"",E77&lt;&gt;""),E77-D77,"")</f>
+        <f>IF(AND(D77&lt;&gt;"",E77&lt;&gt;""),INT(E77)-INT(D77),"")</f>
         <v/>
       </c>
       <c r="G77" s="30" t="inlineStr">
@@ -6205,7 +6205,7 @@
       <c r="D78" s="51" t="n"/>
       <c r="E78" s="51" t="n"/>
       <c r="F78" s="13">
-        <f>IF(AND(D78&lt;&gt;"",E78&lt;&gt;""),E78-D78,"")</f>
+        <f>IF(AND(D78&lt;&gt;"",E78&lt;&gt;""),INT(E78)-INT(D78),"")</f>
         <v/>
       </c>
       <c r="G78" s="24" t="inlineStr">
@@ -6269,7 +6269,7 @@
       <c r="D79" s="53" t="n"/>
       <c r="E79" s="53" t="n"/>
       <c r="F79" s="18">
-        <f>IF(AND(D79&lt;&gt;"",E79&lt;&gt;""),E79-D79,"")</f>
+        <f>IF(AND(D79&lt;&gt;"",E79&lt;&gt;""),INT(E79)-INT(D79),"")</f>
         <v/>
       </c>
       <c r="G79" s="30" t="inlineStr">
@@ -6333,7 +6333,7 @@
       <c r="D80" s="51" t="n"/>
       <c r="E80" s="51" t="n"/>
       <c r="F80" s="13">
-        <f>IF(AND(D80&lt;&gt;"",E80&lt;&gt;""),E80-D80,"")</f>
+        <f>IF(AND(D80&lt;&gt;"",E80&lt;&gt;""),INT(E80)-INT(D80),"")</f>
         <v/>
       </c>
       <c r="G80" s="24" t="inlineStr">
@@ -6397,7 +6397,7 @@
       <c r="D81" s="53" t="n"/>
       <c r="E81" s="53" t="n"/>
       <c r="F81" s="18">
-        <f>IF(AND(D81&lt;&gt;"",E81&lt;&gt;""),E81-D81,"")</f>
+        <f>IF(AND(D81&lt;&gt;"",E81&lt;&gt;""),INT(E81)-INT(D81),"")</f>
         <v/>
       </c>
       <c r="G81" s="30" t="inlineStr">
@@ -6461,7 +6461,7 @@
       <c r="D82" s="51" t="n"/>
       <c r="E82" s="51" t="n"/>
       <c r="F82" s="13">
-        <f>IF(AND(D82&lt;&gt;"",E82&lt;&gt;""),E82-D82,"")</f>
+        <f>IF(AND(D82&lt;&gt;"",E82&lt;&gt;""),INT(E82)-INT(D82),"")</f>
         <v/>
       </c>
       <c r="G82" s="24" t="inlineStr">
@@ -6525,7 +6525,7 @@
       <c r="D83" s="53" t="n"/>
       <c r="E83" s="53" t="n"/>
       <c r="F83" s="18">
-        <f>IF(AND(D83&lt;&gt;"",E83&lt;&gt;""),E83-D83,"")</f>
+        <f>IF(AND(D83&lt;&gt;"",E83&lt;&gt;""),INT(E83)-INT(D83),"")</f>
         <v/>
       </c>
       <c r="G83" s="30" t="inlineStr">
@@ -6589,7 +6589,7 @@
       <c r="D84" s="51" t="n"/>
       <c r="E84" s="51" t="n"/>
       <c r="F84" s="13">
-        <f>IF(AND(D84&lt;&gt;"",E84&lt;&gt;""),E84-D84,"")</f>
+        <f>IF(AND(D84&lt;&gt;"",E84&lt;&gt;""),INT(E84)-INT(D84),"")</f>
         <v/>
       </c>
       <c r="G84" s="24" t="inlineStr">
@@ -6653,7 +6653,7 @@
       <c r="D85" s="53" t="n"/>
       <c r="E85" s="53" t="n"/>
       <c r="F85" s="18">
-        <f>IF(AND(D85&lt;&gt;"",E85&lt;&gt;""),E85-D85,"")</f>
+        <f>IF(AND(D85&lt;&gt;"",E85&lt;&gt;""),INT(E85)-INT(D85),"")</f>
         <v/>
       </c>
       <c r="G85" s="30" t="inlineStr">
@@ -6717,7 +6717,7 @@
       <c r="D86" s="51" t="n"/>
       <c r="E86" s="51" t="n"/>
       <c r="F86" s="13">
-        <f>IF(AND(D86&lt;&gt;"",E86&lt;&gt;""),E86-D86,"")</f>
+        <f>IF(AND(D86&lt;&gt;"",E86&lt;&gt;""),INT(E86)-INT(D86),"")</f>
         <v/>
       </c>
       <c r="G86" s="24" t="inlineStr">
@@ -6781,7 +6781,7 @@
       <c r="D87" s="53" t="n"/>
       <c r="E87" s="53" t="n"/>
       <c r="F87" s="18">
-        <f>IF(AND(D87&lt;&gt;"",E87&lt;&gt;""),E87-D87,"")</f>
+        <f>IF(AND(D87&lt;&gt;"",E87&lt;&gt;""),INT(E87)-INT(D87),"")</f>
         <v/>
       </c>
       <c r="G87" s="30" t="inlineStr">
@@ -6845,7 +6845,7 @@
       <c r="D88" s="51" t="n"/>
       <c r="E88" s="51" t="n"/>
       <c r="F88" s="13">
-        <f>IF(AND(D88&lt;&gt;"",E88&lt;&gt;""),E88-D88,"")</f>
+        <f>IF(AND(D88&lt;&gt;"",E88&lt;&gt;""),INT(E88)-INT(D88),"")</f>
         <v/>
       </c>
       <c r="G88" s="24" t="inlineStr">
@@ -6909,7 +6909,7 @@
       <c r="D89" s="53" t="n"/>
       <c r="E89" s="53" t="n"/>
       <c r="F89" s="18">
-        <f>IF(AND(D89&lt;&gt;"",E89&lt;&gt;""),E89-D89,"")</f>
+        <f>IF(AND(D89&lt;&gt;"",E89&lt;&gt;""),INT(E89)-INT(D89),"")</f>
         <v/>
       </c>
       <c r="G89" s="30" t="inlineStr">
@@ -6973,7 +6973,7 @@
       <c r="D90" s="51" t="n"/>
       <c r="E90" s="51" t="n"/>
       <c r="F90" s="13">
-        <f>IF(AND(D90&lt;&gt;"",E90&lt;&gt;""),E90-D90,"")</f>
+        <f>IF(AND(D90&lt;&gt;"",E90&lt;&gt;""),INT(E90)-INT(D90),"")</f>
         <v/>
       </c>
       <c r="G90" s="24" t="inlineStr">
@@ -7037,7 +7037,7 @@
       <c r="D91" s="53" t="n"/>
       <c r="E91" s="53" t="n"/>
       <c r="F91" s="18">
-        <f>IF(AND(D91&lt;&gt;"",E91&lt;&gt;""),E91-D91,"")</f>
+        <f>IF(AND(D91&lt;&gt;"",E91&lt;&gt;""),INT(E91)-INT(D91),"")</f>
         <v/>
       </c>
       <c r="G91" s="30" t="inlineStr">
@@ -7101,7 +7101,7 @@
       <c r="D92" s="51" t="n"/>
       <c r="E92" s="51" t="n"/>
       <c r="F92" s="13">
-        <f>IF(AND(D92&lt;&gt;"",E92&lt;&gt;""),E92-D92,"")</f>
+        <f>IF(AND(D92&lt;&gt;"",E92&lt;&gt;""),INT(E92)-INT(D92),"")</f>
         <v/>
       </c>
       <c r="G92" s="24" t="inlineStr">
@@ -7165,7 +7165,7 @@
       <c r="D93" s="53" t="n"/>
       <c r="E93" s="53" t="n"/>
       <c r="F93" s="18">
-        <f>IF(AND(D93&lt;&gt;"",E93&lt;&gt;""),E93-D93,"")</f>
+        <f>IF(AND(D93&lt;&gt;"",E93&lt;&gt;""),INT(E93)-INT(D93),"")</f>
         <v/>
       </c>
       <c r="G93" s="30" t="inlineStr">
@@ -7229,7 +7229,7 @@
       <c r="D94" s="51" t="n"/>
       <c r="E94" s="51" t="n"/>
       <c r="F94" s="13">
-        <f>IF(AND(D94&lt;&gt;"",E94&lt;&gt;""),E94-D94,"")</f>
+        <f>IF(AND(D94&lt;&gt;"",E94&lt;&gt;""),INT(E94)-INT(D94),"")</f>
         <v/>
       </c>
       <c r="G94" s="24" t="inlineStr">
@@ -7293,7 +7293,7 @@
       <c r="D95" s="53" t="n"/>
       <c r="E95" s="53" t="n"/>
       <c r="F95" s="18">
-        <f>IF(AND(D95&lt;&gt;"",E95&lt;&gt;""),E95-D95,"")</f>
+        <f>IF(AND(D95&lt;&gt;"",E95&lt;&gt;""),INT(E95)-INT(D95),"")</f>
         <v/>
       </c>
       <c r="G95" s="30" t="inlineStr">
@@ -7357,7 +7357,7 @@
       <c r="D96" s="51" t="n"/>
       <c r="E96" s="51" t="n"/>
       <c r="F96" s="13">
-        <f>IF(AND(D96&lt;&gt;"",E96&lt;&gt;""),E96-D96,"")</f>
+        <f>IF(AND(D96&lt;&gt;"",E96&lt;&gt;""),INT(E96)-INT(D96),"")</f>
         <v/>
       </c>
       <c r="G96" s="24" t="inlineStr">
@@ -7421,7 +7421,7 @@
       <c r="D97" s="53" t="n"/>
       <c r="E97" s="53" t="n"/>
       <c r="F97" s="18">
-        <f>IF(AND(D97&lt;&gt;"",E97&lt;&gt;""),E97-D97,"")</f>
+        <f>IF(AND(D97&lt;&gt;"",E97&lt;&gt;""),INT(E97)-INT(D97),"")</f>
         <v/>
       </c>
       <c r="G97" s="30" t="inlineStr">
@@ -7485,7 +7485,7 @@
       <c r="D98" s="51" t="n"/>
       <c r="E98" s="51" t="n"/>
       <c r="F98" s="13">
-        <f>IF(AND(D98&lt;&gt;"",E98&lt;&gt;""),E98-D98,"")</f>
+        <f>IF(AND(D98&lt;&gt;"",E98&lt;&gt;""),INT(E98)-INT(D98),"")</f>
         <v/>
       </c>
       <c r="G98" s="24" t="inlineStr">
@@ -7549,7 +7549,7 @@
       <c r="D99" s="53" t="n"/>
       <c r="E99" s="53" t="n"/>
       <c r="F99" s="18">
-        <f>IF(AND(D99&lt;&gt;"",E99&lt;&gt;""),E99-D99,"")</f>
+        <f>IF(AND(D99&lt;&gt;"",E99&lt;&gt;""),INT(E99)-INT(D99),"")</f>
         <v/>
       </c>
       <c r="G99" s="30" t="inlineStr">
@@ -7617,7 +7617,7 @@
       <c r="D100" s="51" t="n"/>
       <c r="E100" s="51" t="n"/>
       <c r="F100" s="13">
-        <f>IF(AND(D100&lt;&gt;"",E100&lt;&gt;""),E100-D100,"")</f>
+        <f>IF(AND(D100&lt;&gt;"",E100&lt;&gt;""),INT(E100)-INT(D100),"")</f>
         <v/>
       </c>
       <c r="G100" s="24" t="inlineStr">
@@ -7685,7 +7685,7 @@
       <c r="D101" s="53" t="n"/>
       <c r="E101" s="53" t="n"/>
       <c r="F101" s="18">
-        <f>IF(AND(D101&lt;&gt;"",E101&lt;&gt;""),E101-D101,"")</f>
+        <f>IF(AND(D101&lt;&gt;"",E101&lt;&gt;""),INT(E101)-INT(D101),"")</f>
         <v/>
       </c>
       <c r="G101" s="30" t="inlineStr">
@@ -7753,7 +7753,7 @@
       <c r="D102" s="51" t="n"/>
       <c r="E102" s="51" t="n"/>
       <c r="F102" s="13">
-        <f>IF(AND(D102&lt;&gt;"",E102&lt;&gt;""),E102-D102,"")</f>
+        <f>IF(AND(D102&lt;&gt;"",E102&lt;&gt;""),INT(E102)-INT(D102),"")</f>
         <v/>
       </c>
       <c r="G102" s="24" t="inlineStr">
@@ -7821,7 +7821,7 @@
       <c r="D103" s="53" t="n"/>
       <c r="E103" s="53" t="n"/>
       <c r="F103" s="18">
-        <f>IF(AND(D103&lt;&gt;"",E103&lt;&gt;""),E103-D103,"")</f>
+        <f>IF(AND(D103&lt;&gt;"",E103&lt;&gt;""),INT(E103)-INT(D103),"")</f>
         <v/>
       </c>
       <c r="G103" s="30" t="inlineStr">
@@ -7889,7 +7889,7 @@
       <c r="D104" s="51" t="n"/>
       <c r="E104" s="51" t="n"/>
       <c r="F104" s="13">
-        <f>IF(AND(D104&lt;&gt;"",E104&lt;&gt;""),E104-D104,"")</f>
+        <f>IF(AND(D104&lt;&gt;"",E104&lt;&gt;""),INT(E104)-INT(D104),"")</f>
         <v/>
       </c>
       <c r="G104" s="24" t="inlineStr">
@@ -7957,7 +7957,7 @@
       <c r="D105" s="53" t="n"/>
       <c r="E105" s="53" t="n"/>
       <c r="F105" s="18">
-        <f>IF(AND(D105&lt;&gt;"",E105&lt;&gt;""),E105-D105,"")</f>
+        <f>IF(AND(D105&lt;&gt;"",E105&lt;&gt;""),INT(E105)-INT(D105),"")</f>
         <v/>
       </c>
       <c r="G105" s="30" t="inlineStr">
@@ -8025,7 +8025,7 @@
       <c r="D106" s="51" t="n"/>
       <c r="E106" s="51" t="n"/>
       <c r="F106" s="13">
-        <f>IF(AND(D106&lt;&gt;"",E106&lt;&gt;""),E106-D106,"")</f>
+        <f>IF(AND(D106&lt;&gt;"",E106&lt;&gt;""),INT(E106)-INT(D106),"")</f>
         <v/>
       </c>
       <c r="G106" s="24" t="inlineStr">
@@ -8093,7 +8093,7 @@
       <c r="D107" s="53" t="n"/>
       <c r="E107" s="53" t="n"/>
       <c r="F107" s="18">
-        <f>IF(AND(D107&lt;&gt;"",E107&lt;&gt;""),E107-D107,"")</f>
+        <f>IF(AND(D107&lt;&gt;"",E107&lt;&gt;""),INT(E107)-INT(D107),"")</f>
         <v/>
       </c>
       <c r="G107" s="30" t="inlineStr">
@@ -8157,7 +8157,7 @@
       <c r="D108" s="51" t="n"/>
       <c r="E108" s="51" t="n"/>
       <c r="F108" s="13">
-        <f>IF(AND(D108&lt;&gt;"",E108&lt;&gt;""),E108-D108,"")</f>
+        <f>IF(AND(D108&lt;&gt;"",E108&lt;&gt;""),INT(E108)-INT(D108),"")</f>
         <v/>
       </c>
       <c r="G108" s="24" t="inlineStr">
@@ -8221,7 +8221,7 @@
       <c r="D109" s="53" t="n"/>
       <c r="E109" s="53" t="n"/>
       <c r="F109" s="18">
-        <f>IF(AND(D109&lt;&gt;"",E109&lt;&gt;""),E109-D109,"")</f>
+        <f>IF(AND(D109&lt;&gt;"",E109&lt;&gt;""),INT(E109)-INT(D109),"")</f>
         <v/>
       </c>
       <c r="G109" s="30" t="inlineStr">
@@ -8285,7 +8285,7 @@
       <c r="D110" s="51" t="n"/>
       <c r="E110" s="51" t="n"/>
       <c r="F110" s="13">
-        <f>IF(AND(D110&lt;&gt;"",E110&lt;&gt;""),E110-D110,"")</f>
+        <f>IF(AND(D110&lt;&gt;"",E110&lt;&gt;""),INT(E110)-INT(D110),"")</f>
         <v/>
       </c>
       <c r="G110" s="24" t="inlineStr">
@@ -8349,7 +8349,7 @@
       <c r="D111" s="53" t="n"/>
       <c r="E111" s="53" t="n"/>
       <c r="F111" s="18">
-        <f>IF(AND(D111&lt;&gt;"",E111&lt;&gt;""),E111-D111,"")</f>
+        <f>IF(AND(D111&lt;&gt;"",E111&lt;&gt;""),INT(E111)-INT(D111),"")</f>
         <v/>
       </c>
       <c r="G111" s="30" t="inlineStr">
@@ -8413,7 +8413,7 @@
       <c r="D112" s="51" t="n"/>
       <c r="E112" s="51" t="n"/>
       <c r="F112" s="13">
-        <f>IF(AND(D112&lt;&gt;"",E112&lt;&gt;""),E112-D112,"")</f>
+        <f>IF(AND(D112&lt;&gt;"",E112&lt;&gt;""),INT(E112)-INT(D112),"")</f>
         <v/>
       </c>
       <c r="G112" s="24" t="inlineStr">
@@ -8477,7 +8477,7 @@
       <c r="D113" s="53" t="n"/>
       <c r="E113" s="53" t="n"/>
       <c r="F113" s="18">
-        <f>IF(AND(D113&lt;&gt;"",E113&lt;&gt;""),E113-D113,"")</f>
+        <f>IF(AND(D113&lt;&gt;"",E113&lt;&gt;""),INT(E113)-INT(D113),"")</f>
         <v/>
       </c>
       <c r="G113" s="30" t="inlineStr">
@@ -8541,7 +8541,7 @@
       <c r="D114" s="51" t="n"/>
       <c r="E114" s="51" t="n"/>
       <c r="F114" s="13">
-        <f>IF(AND(D114&lt;&gt;"",E114&lt;&gt;""),E114-D114,"")</f>
+        <f>IF(AND(D114&lt;&gt;"",E114&lt;&gt;""),INT(E114)-INT(D114),"")</f>
         <v/>
       </c>
       <c r="G114" s="24" t="inlineStr">
@@ -8605,7 +8605,7 @@
       <c r="D115" s="53" t="n"/>
       <c r="E115" s="53" t="n"/>
       <c r="F115" s="18">
-        <f>IF(AND(D115&lt;&gt;"",E115&lt;&gt;""),E115-D115,"")</f>
+        <f>IF(AND(D115&lt;&gt;"",E115&lt;&gt;""),INT(E115)-INT(D115),"")</f>
         <v/>
       </c>
       <c r="G115" s="30" t="inlineStr">
@@ -8669,7 +8669,7 @@
       <c r="D116" s="51" t="n"/>
       <c r="E116" s="51" t="n"/>
       <c r="F116" s="13">
-        <f>IF(AND(D116&lt;&gt;"",E116&lt;&gt;""),E116-D116,"")</f>
+        <f>IF(AND(D116&lt;&gt;"",E116&lt;&gt;""),INT(E116)-INT(D116),"")</f>
         <v/>
       </c>
       <c r="G116" s="24" t="inlineStr">
@@ -8733,7 +8733,7 @@
       <c r="D117" s="53" t="n"/>
       <c r="E117" s="53" t="n"/>
       <c r="F117" s="18">
-        <f>IF(AND(D117&lt;&gt;"",E117&lt;&gt;""),E117-D117,"")</f>
+        <f>IF(AND(D117&lt;&gt;"",E117&lt;&gt;""),INT(E117)-INT(D117),"")</f>
         <v/>
       </c>
       <c r="G117" s="30" t="inlineStr">
@@ -8797,7 +8797,7 @@
       <c r="D118" s="51" t="n"/>
       <c r="E118" s="51" t="n"/>
       <c r="F118" s="13">
-        <f>IF(AND(D118&lt;&gt;"",E118&lt;&gt;""),E118-D118,"")</f>
+        <f>IF(AND(D118&lt;&gt;"",E118&lt;&gt;""),INT(E118)-INT(D118),"")</f>
         <v/>
       </c>
       <c r="G118" s="24" t="inlineStr">
@@ -8861,7 +8861,7 @@
       <c r="D119" s="53" t="n"/>
       <c r="E119" s="53" t="n"/>
       <c r="F119" s="18">
-        <f>IF(AND(D119&lt;&gt;"",E119&lt;&gt;""),E119-D119,"")</f>
+        <f>IF(AND(D119&lt;&gt;"",E119&lt;&gt;""),INT(E119)-INT(D119),"")</f>
         <v/>
       </c>
       <c r="G119" s="30" t="inlineStr">
@@ -8925,7 +8925,7 @@
       <c r="D120" s="51" t="n"/>
       <c r="E120" s="51" t="n"/>
       <c r="F120" s="13">
-        <f>IF(AND(D120&lt;&gt;"",E120&lt;&gt;""),E120-D120,"")</f>
+        <f>IF(AND(D120&lt;&gt;"",E120&lt;&gt;""),INT(E120)-INT(D120),"")</f>
         <v/>
       </c>
       <c r="G120" s="24" t="inlineStr">
@@ -8989,7 +8989,7 @@
       <c r="D121" s="53" t="n"/>
       <c r="E121" s="53" t="n"/>
       <c r="F121" s="18">
-        <f>IF(AND(D121&lt;&gt;"",E121&lt;&gt;""),E121-D121,"")</f>
+        <f>IF(AND(D121&lt;&gt;"",E121&lt;&gt;""),INT(E121)-INT(D121),"")</f>
         <v/>
       </c>
       <c r="G121" s="30" t="inlineStr">
@@ -9053,7 +9053,7 @@
       <c r="D122" s="51" t="n"/>
       <c r="E122" s="51" t="n"/>
       <c r="F122" s="13">
-        <f>IF(AND(D122&lt;&gt;"",E122&lt;&gt;""),E122-D122,"")</f>
+        <f>IF(AND(D122&lt;&gt;"",E122&lt;&gt;""),INT(E122)-INT(D122),"")</f>
         <v/>
       </c>
       <c r="G122" s="24" t="inlineStr">
@@ -9117,7 +9117,7 @@
       <c r="D123" s="53" t="n"/>
       <c r="E123" s="53" t="n"/>
       <c r="F123" s="18">
-        <f>IF(AND(D123&lt;&gt;"",E123&lt;&gt;""),E123-D123,"")</f>
+        <f>IF(AND(D123&lt;&gt;"",E123&lt;&gt;""),INT(E123)-INT(D123),"")</f>
         <v/>
       </c>
       <c r="G123" s="30" t="inlineStr">

</xml_diff>